<commit_message>
Lit review page: two-column overview, method description combined, template method and data_source wording matched
</commit_message>
<xml_diff>
--- a/assets/files/lit-review-matrix-template.xlsx
+++ b/assets/files/lit-review-matrix-template.xlsx
@@ -680,7 +680,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>The empirical method. In applied microeconomics this is typically the identification strategy: panel data with fixed effects, instrumental variables, a natural experiment, regression discontinuity, a randomized trial</t>
+          <t>The identification strategy: fixed effects, instrumental variables, regression discontinuity, a natural experiment, or a randomized trial (for a trial, describe the treatment)</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>The named datasets: a Demographic and Health Survey, a census, administrative records, or the authors' own survey</t>
+          <t>The datasets: a Demographic and Health Survey, a census, administrative records, or the authors' own survey</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ etjernst/etjernst.github.io@2b9a0dd6f7760c0749f56930e9eb67a83e83c5d2 🚀
</commit_message>
<xml_diff>
--- a/assets/files/lit-review-matrix-template.xlsx
+++ b/assets/files/lit-review-matrix-template.xlsx
@@ -680,7 +680,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>The empirical method. In applied microeconomics this is typically the identification strategy: panel data with fixed effects, instrumental variables, a natural experiment, regression discontinuity, a randomized trial</t>
+          <t>The identification strategy: fixed effects, instrumental variables, regression discontinuity, a natural experiment, or a randomized trial (for a trial, describe the treatment)</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>The named datasets: a Demographic and Health Survey, a census, administrative records, or the authors' own survey</t>
+          <t>The datasets: a Demographic and Health Survey, a census, administrative records, or the authors' own survey</t>
         </is>
       </c>
     </row>

</xml_diff>